<commit_message>
corpus(rs2-66): every soft band is meshed at the vendor's own density
_rs2_66_slope_data now writes a mesh refinement polygon over the soft stratum at
1.05 m, and rs2_66a-e are rebuilt from it. Both mechanisms of this problem run
through that band, and at the family's 3 m global size it carried about one
element row (115 elements across the h1 = 2 m band at 2.284 m, against RS2's own
508 at 1.087 m), which left the deep factor of safety following node placement
rather than refinement: 1.169, 1.269, 1.106, 1.106 at global 4, 3, 2.2 and 1.5 m.
At the vendor's density it holds still -- 1.131 at global 4 and 3 m, 1.144 at
2.2 m. verify_rebuild --group rs2 reproduces all 57 targets, the five 66 files
included; no other corpus file moves.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/rs2_66a.xlsx
+++ b/docs/verification/files/rocscience/rs2_66a.xlsx
@@ -8853,7 +8853,7 @@
       </c>
       <c r="K5" s="39" t="inlineStr">
         <is>
-          <t>material</t>
+          <t>refine</t>
         </is>
       </c>
       <c r="M5" s="58" t="inlineStr">
@@ -9005,9 +9005,7 @@
           <t>Mat ID:</t>
         </is>
       </c>
-      <c r="K6" s="39" t="n">
-        <v>4</v>
-      </c>
+      <c r="K6" s="39"/>
       <c r="M6" s="58" t="inlineStr">
         <is>
           <t>Mat ID:</t>
@@ -9214,7 +9212,9 @@
           <t>Size:</t>
         </is>
       </c>
-      <c r="K8" s="39" t="n"/>
+      <c r="K8" s="39">
+        <v>1.05</v>
+      </c>
       <c r="M8" s="58" t="inlineStr">
         <is>
           <t>Size:</t>
@@ -9469,8 +9469,12 @@
       <c r="H10" s="3">
         <v>0.0</v>
       </c>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
+      <c r="J10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K10" s="3">
+        <v>10.0</v>
+      </c>
       <c r="M10" s="3" t="n"/>
       <c r="N10" s="3" t="n"/>
       <c r="P10" s="3" t="n"/>
@@ -9521,8 +9525,12 @@
       <c r="H11" s="3">
         <v>0.0</v>
       </c>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
+      <c r="J11" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="K11" s="3">
+        <v>10.0</v>
+      </c>
       <c r="M11" s="3" t="n"/>
       <c r="N11" s="3" t="n"/>
       <c r="P11" s="3" t="n"/>
@@ -9573,8 +9581,12 @@
       <c r="H12" s="3">
         <v>10.0</v>
       </c>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
+      <c r="J12" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="K12" s="3">
+        <v>12.0</v>
+      </c>
       <c r="M12" s="3" t="n"/>
       <c r="N12" s="3" t="n"/>
       <c r="P12" s="3" t="n"/>
@@ -9625,8 +9637,12 @@
       <c r="H13" s="3">
         <v>10.0</v>
       </c>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
+      <c r="J13" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K13" s="3">
+        <v>12.0</v>
+      </c>
       <c r="M13" s="3" t="n"/>
       <c r="N13" s="3" t="n"/>
       <c r="P13" s="3" t="n"/>

</xml_diff>